<commit_message>
Making files realistic - gpt56terra
</commit_message>
<xml_diff>
--- a/MyBudget.OperationsLoading.Tests/Resources/BNP_TestOperations_2026_04.xlsx
+++ b/MyBudget.OperationsLoading.Tests/Resources/BNP_TestOperations_2026_04.xlsx
@@ -448,14 +448,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2">
         <v>46113</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2">
         <v>46113</v>
       </c>
       <c r="D2">
-        <v>5500.00</v>
+        <v>6900.00</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -464,12 +464,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pracodawca</t>
+          <t>Pracodawca Anny Nowak</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Wynagrodzenie Anna Nowak</t>
+          <t>Przelew wynagrodzenia - Anna Nowak</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="K2">
-        <v>5500.00</v>
+        <v>6900.00</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -496,30 +496,33 @@
           <t>Zrealizowana</t>
         </is>
       </c>
+      <c r="N2">
+        <v>10250.00</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3">
         <v>46114</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3">
         <v>46114</v>
       </c>
       <c r="D3">
-        <v>4200.00</v>
+        <v>-2661.20</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>PLN</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Pracodawca</t>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wspólnota Mieszkaniowa Zielone Tarasy</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Wynagrodzenie Piotr Nowak</t>
+          <t>Czynsz za mieszkanie</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -530,11 +533,11 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>PRZELEW PRZYCHODZĄCY</t>
+          <t>PRZELEW WYKONANY</t>
         </is>
       </c>
       <c r="K3">
-        <v>4200.00</v>
+        <v>-2661.20</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -546,16 +549,19 @@
           <t>Zrealizowana</t>
         </is>
       </c>
+      <c r="N3">
+        <v>7588.80</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4">
         <v>46115</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4">
         <v>46115</v>
       </c>
       <c r="D4">
-        <v>-2800.00</v>
+        <v>-499.00</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -564,12 +570,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Wspólnota</t>
+          <t>Biedronka</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Czynsz</t>
+          <t>Zakupy spożywcze dla rodziny</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -580,371 +586,395 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>PŁATNOŚĆ KARTĄ</t>
+        </is>
+      </c>
+      <c r="K4">
+        <v>-499.00</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Zrealizowana</t>
+        </is>
+      </c>
+      <c r="N4">
+        <v>7089.80</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>46116</v>
+      </c>
+      <c r="B5">
+        <v>46116</v>
+      </c>
+      <c r="D5">
+        <v>-793.40</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Przedszkole Słoneczko</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Czesne za przedszkole</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Konto Osobiste
+00203000450000123456789000</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>PRZELEW WYKONANY</t>
         </is>
       </c>
-      <c r="K4">
-        <v>-2800.00</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
+      <c r="K5">
+        <v>-793.40</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Zrealizowana</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>46116</v>
-      </c>
-      <c r="B5" s="4">
-        <v>46116</v>
-      </c>
-      <c r="D5">
-        <v>-533.70</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Lidl</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Lidl</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="N5">
+        <v>6296.40</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>46117</v>
+      </c>
+      <c r="B6">
+        <v>46117</v>
+      </c>
+      <c r="D6">
+        <v>-176.10</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Smyk</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Artykuły dla dzieci</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Konto Osobiste
 00203000450000123456789000</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>PŁATNOŚĆ KARTĄ</t>
         </is>
       </c>
-      <c r="K5">
-        <v>-533.70</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
+      <c r="K6">
+        <v>-176.10</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Zrealizowana</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>46117</v>
-      </c>
-      <c r="B6" s="4">
-        <v>46117</v>
-      </c>
-      <c r="D6">
-        <v>-198.50</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Orlen</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Orlen</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="N6">
+        <v>6120.30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>46118</v>
+      </c>
+      <c r="B7">
+        <v>46118</v>
+      </c>
+      <c r="D7">
+        <v>-144.70</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Rossmann</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Chemia domowa i kosmetyki</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Konto Osobiste
 00203000450000123456789000</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>PŁATNOŚĆ KARTĄ</t>
         </is>
       </c>
-      <c r="K6">
-        <v>-198.50</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+      <c r="K7">
+        <v>-144.70</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>Zrealizowana</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>46118</v>
-      </c>
-      <c r="B7" s="4">
-        <v>46118</v>
-      </c>
-      <c r="D7">
-        <v>-89.99</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="N7">
+        <v>5975.60</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>46119</v>
+      </c>
+      <c r="B8">
+        <v>46119</v>
+      </c>
+      <c r="D8">
+        <v>-110.20</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Apteka Dr.Max</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Leki dla rodziny</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Konto Osobiste
+00203000450000123456789000</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PŁATNOŚĆ KARTĄ</t>
+        </is>
+      </c>
+      <c r="K8">
+        <v>-110.20</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Zrealizowana</t>
+        </is>
+      </c>
+      <c r="N8">
+        <v>5865.40</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>46120</v>
+      </c>
+      <c r="B9">
+        <v>46120</v>
+      </c>
+      <c r="D9">
+        <v>-229.70</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Zara</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ubrania dziecięce</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Konto Osobiste
+00203000450000123456789000</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PŁATNOŚĆ KARTĄ</t>
+        </is>
+      </c>
+      <c r="K9">
+        <v>-229.70</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Zrealizowana</t>
+        </is>
+      </c>
+      <c r="N9">
+        <v>5635.70</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>46121</v>
+      </c>
+      <c r="B10">
+        <v>46121</v>
+      </c>
+      <c r="D10">
+        <v>-86.29</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Empik</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Empik</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Książki i materiały szkolne</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Konto Osobiste
 00203000450000123456789000</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>PŁATNOŚĆ KARTĄ</t>
         </is>
       </c>
-      <c r="K7">
-        <v>-89.99</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
+      <c r="K10">
+        <v>-86.29</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Zrealizowana</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>46119</v>
-      </c>
-      <c r="B8" s="4">
-        <v>46119</v>
-      </c>
-      <c r="D8">
-        <v>-210.00</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="N10">
+        <v>5549.41</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>46122</v>
+      </c>
+      <c r="B11">
+        <v>46122</v>
+      </c>
+      <c r="D11">
+        <v>-371.70</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Biedronka</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Zakupy spożywcze - weekend</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Konto Osobiste
 00203000450000123456789000</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>PRZELEW WYKONANY</t>
-        </is>
-      </c>
-      <c r="K8">
-        <v>-210.00</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>PŁATNOŚĆ KARTĄ</t>
+        </is>
+      </c>
+      <c r="K11">
+        <v>-371.70</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Zrealizowana</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>46120</v>
-      </c>
-      <c r="B9" s="4">
-        <v>46120</v>
-      </c>
-      <c r="D9">
-        <v>-76.40</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Apteka</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Apteka</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Konto Osobiste
-00203000450000123456789000</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>PŁATNOŚĆ KARTĄ</t>
-        </is>
-      </c>
-      <c r="K9">
-        <v>-76.40</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Zrealizowana</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>46121</v>
-      </c>
-      <c r="B10" s="4">
-        <v>46121</v>
-      </c>
-      <c r="D10">
-        <v>-340.00</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Przedszkole</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Przedszkole</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Konto Osobiste
-00203000450000123456789000</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>PRZELEW WYKONANY</t>
-        </is>
-      </c>
-      <c r="K10">
-        <v>-340.00</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Zrealizowana</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4">
-        <v>46122</v>
-      </c>
-      <c r="B11" s="4">
-        <v>46122</v>
-      </c>
-      <c r="D11">
-        <v>-142.30</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Pepco</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Pepco</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Konto Osobiste
-00203000450000123456789000</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>PŁATNOŚĆ KARTĄ</t>
-        </is>
-      </c>
-      <c r="K11">
-        <v>-142.30</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>PLN</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Zrealizowana</t>
-        </is>
+      <c r="N11">
+        <v>5177.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>